<commit_message>
Add Date of birth and Primary PEP role columns to screening list
https://claude.ai/code/session_01KXpyCXhpmrknDcBNv6sDP9
</commit_message>
<xml_diff>
--- a/NBU_Uzbekistan_Board_PEP_Screening.xlsx
+++ b/NBU_Uzbekistan_Board_PEP_Screening.xlsx
@@ -475,19 +475,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +502,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: Decision of the Supervisory Board No. 60 dated 10 December 2025 (Tashkent). Certified English translation. PEP status to be confirmed via screening.</t>
+          <t>Source: Decision of the Supervisory Board No. 60 dated 10 December 2025 (Tashkent). Certified English translation. Date of birth not stated in the document — to be populated during screening. PEP status to be confirmed.</t>
         </is>
       </c>
     </row>
@@ -522,35 +524,45 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Date of birth</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Governance body</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Role at the Bank</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Primary PEP role</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Government / external position (PEP indicator)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Likely PEP category</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Screening status</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Source (page)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -566,37 +578,43 @@
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Chairman of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Minister of Investment, Industry and Trade of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Minister of Investment, Industry and Trade of the Republic of Uzbekistan</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Senior government official (Minister)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Government minister — high PEP relevance.</t>
         </is>
@@ -612,37 +630,43 @@
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Deputy Minister of Economy and Finance of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Minister of Economy and Finance of the Republic of Uzbekistan</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Senior government official (Deputy Minister)</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -654,37 +678,43 @@
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>First Deputy Chairman of the Tax Committee (Cabinet of Ministers of Uzbekistan)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Tax Committee under the Cabinet of Ministers of Uzbekistan</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Senior government official</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -696,37 +726,43 @@
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Head of Legal Service, Reconstruction and Development Fund of Uzbekistan</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Head of Legal Service of the Reconstruction and Development Fund of Uzbekistan</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>State fund official</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -738,33 +774,39 @@
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr">
         <is>
+          <t>Independent director (no government office stated)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
           <t>Possible PEP (verify)</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Independent director.</t>
         </is>
@@ -784,33 +826,39 @@
           <t>Aleksander von Gleich</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
+          <t>Independent director (no government office stated)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
           <t>Foreign national (verify)</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>Name transliterated from Cyrillic; foreign independent director.</t>
         </is>
@@ -830,33 +878,39 @@
           <t>Olivier Grizard</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
+          <t>Independent director (no government office stated)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
           <t>Foreign national (verify)</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Foreign independent director.</t>
         </is>
@@ -872,37 +926,43 @@
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Secretary of the meeting</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Head of Corporate Governance Service (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Head of Corporate Governance Service of the Bank</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Bank officer</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>Meeting secretary; bank staff.</t>
         </is>
@@ -918,37 +978,43 @@
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Chairman of the Board</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Chairman of the Board (CEO) of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Bank executive (CEO-equivalent)</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -960,37 +1026,43 @@
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>First Deputy Chairman of the Board of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1002,37 +1074,43 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Deputy Chairman of the Board of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1044,37 +1122,43 @@
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Chairman of the Board of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1086,37 +1170,43 @@
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Deputy Chairman of the Board of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1128,37 +1218,43 @@
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Chairman of the Board of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1170,37 +1266,43 @@
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board — Director of the Accounting and Reporting Department — Chief Accountant</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Deputy Chairman of the Board / Chief Accountant of a state-owned bank</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Bank executive / Chief Accountant</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1212,37 +1314,43 @@
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Director, Interbank Settlement Center (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Director of the Interbank Settlement Center</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1254,37 +1362,43 @@
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Director, Corporate Relations and Investments Department (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Director of the Corporate Relations and Investments Department</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1296,37 +1410,43 @@
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Director, Administrative Management Department (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Director of the Administrative Management Department</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1342,37 +1462,43 @@
           <t>Nurkulov Sadriddin Jamolovich</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Director, Compliance Risk Unit (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Director of the Compliance Risk Unit</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>p.9-11</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Newly INCLUDED in the Board by this decision.</t>
         </is>
@@ -1392,37 +1518,43 @@
           <t>Kalonov Zokir Botirovich</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Former Management Board member</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>(Excluded) Director of the Department of Administrative Affairs</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Former Director, Department of Administrative Affairs (state-owned bank)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Bank officer (former board member)</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Bank management (former)</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>p.9-10</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>EXCLUDED from the Board by this decision; employment contract terminated.</t>
         </is>
@@ -1430,8 +1562,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Nationality and Passport/ID number columns to screening list
https://claude.ai/code/session_01KXpyCXhpmrknDcBNv6sDP9
</commit_message>
<xml_diff>
--- a/NBU_Uzbekistan_Board_PEP_Screening.xlsx
+++ b/NBU_Uzbekistan_Board_PEP_Screening.xlsx
@@ -475,21 +475,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,40 +531,50 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Nationality</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Passport / ID number</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Governance body</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Role at the Bank</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Primary PEP role</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Government / external position (PEP indicator)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Likely PEP category</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Screening status</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Source (page)</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -579,42 +591,44 @@
       </c>
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Chairman of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Minister of Investment, Industry and Trade of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Minister of Investment, Industry and Trade of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Senior government official (Minister)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Government minister — high PEP relevance.</t>
         </is>
@@ -631,42 +645,44 @@
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Deputy Minister of Economy and Finance of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Deputy Minister of Economy and Finance of the Republic of Uzbekistan</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Senior government official (Deputy Minister)</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -679,42 +695,44 @@
       </c>
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Tax Committee (Cabinet of Ministers of Uzbekistan)</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Tax Committee under the Cabinet of Ministers of Uzbekistan</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Senior government official</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -727,42 +745,44 @@
       </c>
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Head of Legal Service, Reconstruction and Development Fund of Uzbekistan</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Head of Legal Service of the Reconstruction and Development Fund of Uzbekistan</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>State fund official</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -775,38 +795,40 @@
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Independent director (no government office stated)</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Possible PEP (verify)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Independent director.</t>
         </is>
@@ -827,38 +849,40 @@
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Independent director (no government office stated)</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Foreign national (verify)</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>Name transliterated from Cyrillic; foreign independent director.</t>
         </is>
@@ -879,38 +903,40 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Independent Member of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Independent director (no government office stated)</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Foreign national (verify)</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Foreign independent director.</t>
         </is>
@@ -927,42 +953,44 @@
       </c>
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Supervisory Board</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Secretary of the meeting</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Head of Corporate Governance Service (state-owned bank)</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Head of Corporate Governance Service of the Bank</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Bank officer</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>p.9/11</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>Meeting secretary; bank staff.</t>
         </is>
@@ -979,42 +1007,44 @@
       </c>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Chairman of the Board</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Chairman of the Board (CEO) of a state-owned bank</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Bank executive (CEO-equivalent)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1027,42 +1057,44 @@
       </c>
       <c r="C14" s="5" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>First Deputy Chairman of the Board of a state-owned bank</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1075,42 +1107,44 @@
       </c>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board of a state-owned bank</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1123,42 +1157,44 @@
       </c>
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board of a state-owned bank</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1171,42 +1207,44 @@
       </c>
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board of a state-owned bank</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1219,42 +1257,44 @@
       </c>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board of a state-owned bank</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>Bank executive</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1267,42 +1307,44 @@
       </c>
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board — Director of the Accounting and Reporting Department — Chief Accountant</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Deputy Chairman of the Board / Chief Accountant of a state-owned bank</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Bank executive / Chief Accountant</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr"/>
+      <c r="N19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1315,42 +1357,44 @@
       </c>
       <c r="C20" s="5" t="inlineStr"/>
       <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Director, Interbank Settlement Center (state-owned bank)</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Director of the Interbank Settlement Center</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1363,42 +1407,44 @@
       </c>
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Director, Corporate Relations and Investments Department (state-owned bank)</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Director of the Corporate Relations and Investments Department</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr"/>
+      <c r="N21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1411,42 +1457,44 @@
       </c>
       <c r="C22" s="5" t="inlineStr"/>
       <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Director, Administrative Management Department (state-owned bank)</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Director of the Administrative Management Department</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="M22" s="5" t="inlineStr">
         <is>
           <t>p.11</t>
         </is>
       </c>
-      <c r="L22" s="5" t="inlineStr"/>
+      <c r="N22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1463,42 +1511,44 @@
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Management Board</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Member of the Board</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Director, Compliance Risk Unit (state-owned bank)</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Director of the Compliance Risk Unit</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Bank senior management</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>p.9-11</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Newly INCLUDED in the Board by this decision.</t>
         </is>
@@ -1519,42 +1569,44 @@
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Former Management Board member</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>(Excluded) Director of the Department of Administrative Affairs</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Former Director, Department of Administrative Affairs (state-owned bank)</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Bank officer (former board member)</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>Bank management (former)</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>To screen</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="M24" s="5" t="inlineStr">
         <is>
           <t>p.9-10</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>EXCLUDED from the Board by this decision; employment contract terminated.</t>
         </is>
@@ -1562,8 +1614,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>